<commit_message>
Shorten path columns to filenames in Rename Audit tab
</commit_message>
<xml_diff>
--- a/DDL-structure-and-rename-map.xlsx
+++ b/DDL-structure-and-rename-map.xlsx
@@ -9440,12 +9440,12 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Original Path</t>
+          <t>Original Filename</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Current Path</t>
+          <t>Current Filename</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -9477,12 +9477,12 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/4-what-happened-to-anki</t>
+          <t>4-what-happened-to-anki</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>articles/4 - What Happened To Anki.md</t>
+          <t>4 - What Happened To Anki.md</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -9510,12 +9510,12 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/39-vector-or-cozmo-which-one-is-right-for-me</t>
+          <t>39-vector-or-cozmo-which-one-is-right-for-me</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>articles/39 - Vector or Cozmo - Which One Is Right For Me.md</t>
+          <t>39 - Vector or Cozmo - Which One Is Right For Me.md</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -9543,12 +9543,12 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/44-what-do-vectors-back-lights-mean</t>
+          <t>44-what-do-vectors-back-lights-mean</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>articles/44 - What Do Vector's Back Lights Mean.md</t>
+          <t>44 - What Do Vector's Back Lights Mean.md</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -9576,12 +9576,12 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/48-vector-status</t>
+          <t>48-vector-status</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>articles/48 - What is happening with Vector.md</t>
+          <t>48 - What is happening with Vector.md</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -9609,12 +9609,12 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/49-repair-status-vector</t>
+          <t>49-repair-status-vector</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>articles/49 - Do you repair Vectors, Cozmos, or Overdrive Sets.md</t>
+          <t>49 - Do you repair Vectors, Cozmos, or Overdrive Sets.md</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -9642,12 +9642,12 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/54-vector-software-update</t>
+          <t>54-vector-software-update</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>articles/54 - How do I update Vector's software.md</t>
+          <t>54 - How do I update Vector's software.md</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -9675,12 +9675,12 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/83-compatible-devices</t>
+          <t>83-compatible-devices</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>articles/83 - Compatible Devices (Vector).md</t>
+          <t>83 - Compatible Devices (Vector).md</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -9708,12 +9708,12 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/85-compatible-devices-further-information</t>
+          <t>85-compatible-devices-further-information</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>articles/85 - Compatible Devices - Further Information (Vector).md</t>
+          <t>85 - Compatible Devices - Further Information (Vector).md</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -9741,12 +9741,12 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/88-product-disposal-information</t>
+          <t>88-product-disposal-information</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>articles/88 - Product Disposal Information (Vector).md</t>
+          <t>88 - Product Disposal Information (Vector).md</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -9774,12 +9774,12 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/96-vector-status-codes</t>
+          <t>96-vector-status-codes</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>articles/96 - Vector Error &amp; Status Codes.md</t>
+          <t>96 - Vector Error &amp; Status Codes.md</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -9807,12 +9807,12 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/99-vector-does-not-understand-me-troubleshooting-speech-recognition</t>
+          <t>99-vector-does-not-understand-me-troubleshooting-speech-recognition</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>articles/99 - Vector does not understand me - Troubleshooting Speech Recognition.md</t>
+          <t>99 - Vector does not understand me - Troubleshooting Speech Recognition.md</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -9840,12 +9840,12 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/100-troubleshooting-charging-issues</t>
+          <t>100-troubleshooting-charging-issues</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>articles/100 - Troubleshooting Charging Issues.md</t>
+          <t>100 - Troubleshooting Charging Issues.md</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -9873,12 +9873,12 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/101-why-does-vector-show-an-error</t>
+          <t>101-why-does-vector-show-an-error</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>articles/101 - Why does Vector show an error.md</t>
+          <t>101 - Why does Vector show an error.md</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -9906,12 +9906,12 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/102-why-is-there-no-sound</t>
+          <t>102-why-is-there-no-sound</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>articles/102 - Why is there no sound (Vector).md</t>
+          <t>102 - Why is there no sound (Vector).md</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -9939,12 +9939,12 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/103-why-does-vector-need-a-24-ghz-network</t>
+          <t>103-why-does-vector-need-a-24-ghz-network</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>articles/103 - Why does Vector need a 2.4 GHz network.md</t>
+          <t>103 - Why does Vector need a 2.4 GHz network.md</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -9972,12 +9972,12 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/104-troubleshooting-vectore28099s-connection</t>
+          <t>104-troubleshooting-vectore28099s-connection</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>articles/104 - Troubleshooting Vector's Connection.md</t>
+          <t>104 - Troubleshooting Vector's Connection.md</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -10005,12 +10005,12 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/105-vector-security-privacy-faqs</t>
+          <t>105-vector-security-privacy-faqs</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>articles/105 - Vector Security &amp; Privacy FAQs.md</t>
+          <t>105 - Vector Security &amp; Privacy FAQs.md</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -10038,12 +10038,12 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/106-quick-start-guide</t>
+          <t>106-quick-start-guide</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>articles/106 - Quick Start Guide (Vector).md</t>
+          <t>106 - Quick Start Guide (Vector).md</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -10071,12 +10071,12 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/107-product-compliance</t>
+          <t>107-product-compliance</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>articles/107 - Product Compliance (Vector).md</t>
+          <t>107 - Product Compliance (Vector).md</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -10104,12 +10104,12 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/108-vector-changelog-and-known-issues</t>
+          <t>108-vector-changelog-and-known-issues</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>articles/108 - Vector Changelog and Known Issues.md</t>
+          <t>108 - Vector Changelog and Known Issues.md</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -10137,12 +10137,12 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/109-where-can-i-download-the-vector-sdk</t>
+          <t>109-where-can-i-download-the-vector-sdk</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>articles/109 - Where can I download the Vector SDK.md</t>
+          <t>109 - Where can I download the Vector SDK.md</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -10170,12 +10170,12 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/110-integrating-vector-with-amazon-alexa</t>
+          <t>110-integrating-vector-with-amazon-alexa</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>articles/110 - Integrating Vector with Amazon Alexa.md</t>
+          <t>110 - Integrating Vector with Amazon Alexa.md</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -10203,12 +10203,12 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/111-video-vector-and-speech-recognition</t>
+          <t>111-video-vector-and-speech-recognition</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>articles/111 - Vector and Speech Recognition.md</t>
+          <t>111 - Vector and Speech Recognition.md</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -10236,12 +10236,12 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/114-video-vector-and-connection-how-to-set-vector-up</t>
+          <t>114-video-vector-and-connection-how-to-set-vector-up</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>articles/114 - [VIDEO] Vector and Connection - How to set Vector up.md</t>
+          <t>114 - [VIDEO] Vector and Connection - How to set Vector up.md</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -10269,12 +10269,12 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/115-vectore28099s-cube</t>
+          <t>115-vectore28099s-cube</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>articles/115 - Vector’s Cube.md</t>
+          <t>115 - Vector’s Cube.md</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -10302,12 +10302,12 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/116-photos-taken-by-vector</t>
+          <t>116-photos-taken-by-vector</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>articles/116 - Photos taken by Vector.md</t>
+          <t>116 - Photos taken by Vector.md</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -10335,12 +10335,12 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/117-how-to-charge-vector</t>
+          <t>117-how-to-charge-vector</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>articles/117 - How to Charge Vector.md</t>
+          <t>117 - How to Charge Vector.md</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -10368,12 +10368,12 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/118-can-i-use-multiple-vectors-or-devices</t>
+          <t>118-can-i-use-multiple-vectors-or-devices</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>articles/118 - Can I use multiple Vectors or devices.md</t>
+          <t>118 - Can I use multiple Vectors or devices.md</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -10401,12 +10401,12 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/119-how-to-meet-vector</t>
+          <t>119-how-to-meet-vector</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>articles/119 - How to Meet Vector.md</t>
+          <t>119 - How to Meet Vector.md</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -10434,12 +10434,12 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/120-what-do-i-use-the-vector-app-for</t>
+          <t>120-what-do-i-use-the-vector-app-for</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>articles/120 - What do I use the Vector app for.md</t>
+          <t>120 - What do I use the Vector app for.md</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -10467,12 +10467,12 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/121-where-to-use-vector</t>
+          <t>121-where-to-use-vector</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>articles/121 - Where to use Vector.md</t>
+          <t>121 - Where to use Vector.md</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -10500,12 +10500,12 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/122-ways-to-interact-with-vector</t>
+          <t>122-ways-to-interact-with-vector</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>articles/122 - Ways to Interact with Vector.md</t>
+          <t>122 - Ways to Interact with Vector.md</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -10533,12 +10533,12 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/123-updating-your-vector-account</t>
+          <t>123-updating-your-vector-account</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>articles/123 - Updating your Vector account.md</t>
+          <t>123 - Updating your Vector account.md</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -10566,12 +10566,12 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/129-product-disposal-information</t>
+          <t>129-product-disposal-information</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>articles/129 - Product Disposal Information (Cozmo).md</t>
+          <t>129 - Product Disposal Information (Cozmo).md</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -10599,12 +10599,12 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/130-why-do-i-need-a-device</t>
+          <t>130-why-do-i-need-a-device</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>articles/130 - Why do I need a device.md</t>
+          <t>130 - Why do I need a device.md</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -10632,12 +10632,12 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/134-compatible-devices-further-information</t>
+          <t>134-compatible-devices-further-information</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>articles/134 - Compatible Devices - Further Information (Cozmo).md</t>
+          <t>134 - Compatible Devices - Further Information (Cozmo).md</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -10665,12 +10665,12 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/135-compatible-devices</t>
+          <t>135-compatible-devices</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>articles/135 - Compatible Devices (Cozmo).md</t>
+          <t>135 - Compatible Devices (Cozmo).md</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -10698,12 +10698,12 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/139-what-is-the-difference-between-cozmo-and-vector</t>
+          <t>139-what-is-the-difference-between-cozmo-and-vector</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>articles/139 - What is the difference between Cozmo and Vector.md</t>
+          <t>139 - What is the difference between Cozmo and Vector.md</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -10731,12 +10731,12 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/140-where-can-i-purchase-cozmo-cubes-and-other-spare-parts</t>
+          <t>140-where-can-i-purchase-cozmo-cubes-and-other-spare-parts</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>articles/140 - Where can I purchase Cozmo cubes and other spare parts.md</t>
+          <t>140 - Where can I purchase Cozmo cubes and other spare parts.md</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -10764,12 +10764,12 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/209-cozmo-led-summary</t>
+          <t>209-cozmo-led-summary</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>articles/209 - What Do Cozmo's Back Lights Mean.md</t>
+          <t>209 - What Do Cozmo's Back Lights Mean.md</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -10797,12 +10797,12 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/212-why-cant-cozmo-see</t>
+          <t>212-why-cant-cozmo-see</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>articles/212 - Why can't Cozmo see.md</t>
+          <t>212 - Why can't Cozmo see.md</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -10830,12 +10830,12 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/213-why-does-cozmo-not-recognize-me</t>
+          <t>213-why-does-cozmo-not-recognize-me</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>articles/213 - Why does Cozmo not recognize me.md</t>
+          <t>213 - Why does Cozmo not recognize me.md</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
@@ -10863,12 +10863,12 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/214-why-is-there-no-sound</t>
+          <t>214-why-is-there-no-sound</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>articles/214 - Why is there no sound (Cozmo).md</t>
+          <t>214 - Why is there no sound (Cozmo).md</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -10896,12 +10896,12 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/215-is-cozmos-lift-broken</t>
+          <t>215-is-cozmos-lift-broken</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>articles/215 - Is Cozmo's Lift broken.md</t>
+          <t>215 - Is Cozmo's Lift broken.md</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
@@ -10929,12 +10929,12 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/216-why-do-i-see-a-tutorial-paused-error</t>
+          <t>216-why-do-i-see-a-tutorial-paused-error</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>articles/216 - Why do I see a Tutorial Paused error.md</t>
+          <t>216 - Why do I see a Tutorial Paused error.md</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -10962,12 +10962,12 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/217-cant-feed-cozmo</t>
+          <t>217-cant-feed-cozmo</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>articles/217 - Can't Feed Cozmo.md</t>
+          <t>217 - Can't Feed Cozmo.md</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
@@ -10995,12 +10995,12 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/218-why-do-i-get-error-2-error-3</t>
+          <t>218-why-do-i-get-error-2-error-3</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>articles/218 - Why do I get Error 2 - Error 3.md</t>
+          <t>218 - Why do I get Error 2 - Error 3.md</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
@@ -11028,12 +11028,12 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/219-how-to-reset-cozmo-to-factory-firmware</t>
+          <t>219-how-to-reset-cozmo-to-factory-firmware</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>articles/219 - How to reset Cozmo to factory firmware.md</t>
+          <t>219 - How to reset Cozmo to factory firmware.md</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
@@ -11061,12 +11061,12 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/220-how-to-powercycle-cozmo</t>
+          <t>220-how-to-powercycle-cozmo</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>articles/220 - How to powercycle Cozmo.md</t>
+          <t>220 - How to powercycle Cozmo.md</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
@@ -11094,12 +11094,12 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/221-why-does-cozmo-keep-turning-off</t>
+          <t>221-why-does-cozmo-keep-turning-off</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>articles/221 - Why does Cozmo keep turning off.md</t>
+          <t>221 - Why does Cozmo keep turning off.md</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
@@ -11127,12 +11127,12 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/222-cozmos-cubes</t>
+          <t>222-cozmos-cubes</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>articles/222 - Cozmo's Cubes.md</t>
+          <t>222 - Cozmo's Cubes.md</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
@@ -11160,12 +11160,12 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/223-questions-about-cozmos-playtime-and-battery</t>
+          <t>223-questions-about-cozmos-playtime-and-battery</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>articles/223 - Questions about Cozmo's Playtime and Battery.md</t>
+          <t>223 - Questions about Cozmo's Playtime and Battery.md</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
@@ -11193,12 +11193,12 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/224-cozmo-sdk-information</t>
+          <t>224-cozmo-sdk-information</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>articles/224 - Cozmo SDK Information.md</t>
+          <t>224 - Cozmo SDK Information.md</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
@@ -11226,12 +11226,12 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/225-product-compliance</t>
+          <t>225-product-compliance</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>articles/225 - Product Compliance (Cozmo).md</t>
+          <t>225 - Product Compliance (Cozmo).md</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
@@ -11259,12 +11259,12 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/226-cozmo-changelog</t>
+          <t>226-cozmo-changelog</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>articles/226 - Cozmo App Changelog.md</t>
+          <t>226 - Cozmo App Changelog.md</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
@@ -11292,12 +11292,12 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/227-cozmo-privacy-basics</t>
+          <t>227-cozmo-privacy-basics</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>articles/227 - Cozmo Privacy Basics.md</t>
+          <t>227 - Cozmo Privacy Basics.md</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
@@ -11325,12 +11325,12 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/228-download-the-android-kindle-fire-apk</t>
+          <t>228-download-the-android-kindle-fire-apk</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>articles/228 - Download the Android - Kindle Fire APK.md</t>
+          <t>228 - Download the Android - Kindle Fire APK.md</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
@@ -11358,12 +11358,12 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/229-quick-start-guide</t>
+          <t>229-quick-start-guide</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>articles/229 - Quick Start Guide (Cozmo).md</t>
+          <t>229 - Quick Start Guide (Cozmo).md</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
@@ -11391,12 +11391,12 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/230-video-how-do-i-connect-to-cozmoe28099s-wifi-network</t>
+          <t>230-video-how-do-i-connect-to-cozmoe28099s-wifi-network</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>articles/230 - [VIDEO] How do I connect to Cozmo’s WiFi network.md</t>
+          <t>230 - [VIDEO] How do I connect to Cozmo’s WiFi network.md</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
@@ -11424,12 +11424,12 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/231-helpful-tips-to-get-started</t>
+          <t>231-helpful-tips-to-get-started</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>articles/231 - Helpful Tips to Get Started.md</t>
+          <t>231 - Helpful Tips to Get Started.md</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
@@ -11457,12 +11457,12 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/232-how-do-i-turn-off-cozmo</t>
+          <t>232-how-do-i-turn-off-cozmo</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>articles/232 - How do I turn off Cozmo.md</t>
+          <t>232 - How do I turn off Cozmo.md</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
@@ -11490,12 +11490,12 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/233-how-do-i-wake-up-and-reconnect-to-cozmo</t>
+          <t>233-how-do-i-wake-up-and-reconnect-to-cozmo</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>articles/233 - How do I wake up and reconnect to Cozmo.md</t>
+          <t>233 - How do I wake up and reconnect to Cozmo.md</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
@@ -11523,12 +11523,12 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/234-learn-about-code-lab</t>
+          <t>234-learn-about-code-lab</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>articles/234 - Learn about Code Lab.md</t>
+          <t>234 - Learn about Code Lab.md</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
@@ -11556,12 +11556,12 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/235-how-to-charge-cozmo</t>
+          <t>235-how-to-charge-cozmo</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>articles/235 - How to charge Cozmo.md</t>
+          <t>235 - How to charge Cozmo.md</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
@@ -11589,12 +11589,12 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/236-where-to-play-with-cozmo</t>
+          <t>236-where-to-play-with-cozmo</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>articles/236 - Where to play with Cozmo.md</t>
+          <t>236 - Where to play with Cozmo.md</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
@@ -11622,12 +11622,12 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/237-cozmos-needs</t>
+          <t>237-cozmos-needs</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>articles/237 - Cozmo's Needs.md</t>
+          <t>237 - Cozmo's Needs.md</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
@@ -11655,12 +11655,12 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/238-using-cozmo-with-multiple-devices-and-cubes</t>
+          <t>238-using-cozmo-with-multiple-devices-and-cubes</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>articles/238 - Using Cozmo with Multiple Devices and Cubes.md</t>
+          <t>238 - Using Cozmo with Multiple Devices and Cubes.md</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
@@ -11688,12 +11688,12 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/239-what-type-of-laser-pointer-can-i-use-with-cozmo</t>
+          <t>239-what-type-of-laser-pointer-can-i-use-with-cozmo</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>articles/239 - What type of laser pointer can I use with Cozmo.md</t>
+          <t>239 - What type of laser pointer can I use with Cozmo.md</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
@@ -11721,12 +11721,12 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/240-how-to-erase-or-restore-cozmo</t>
+          <t>240-how-to-erase-or-restore-cozmo</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>articles/240 - How to erase or restore Cozmo.md</t>
+          <t>240 - How to erase or restore Cozmo.md</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
@@ -11754,12 +11754,12 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/241-cozmo-and-sparks</t>
+          <t>241-cozmo-and-sparks</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>articles/241 - Cozmo's Sparks.md</t>
+          <t>241 - Cozmo's Sparks.md</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
@@ -11787,12 +11787,12 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/242-learn-more-about-education-edu-mode</t>
+          <t>242-learn-more-about-education-edu-mode</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>articles/242 - Learn more about Education (EDU) Mode.md</t>
+          <t>242 - Learn more about Education (EDU) Mode.md</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
@@ -11820,12 +11820,12 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/243-the-modular-track</t>
+          <t>243-the-modular-track</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>articles/243 - The modular track.md</t>
+          <t>243 - The modular track.md</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
@@ -11853,12 +11853,12 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/244-download-the-android-apk</t>
+          <t>244-download-the-android-apk</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>articles/244 - Download the Drive &amp; OVERDRIVE Android APKs.md</t>
+          <t>244 - Download the Drive &amp; OVERDRIVE Android APKs.md</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
@@ -11886,12 +11886,12 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/245-download-the-kindle-fire-apk</t>
+          <t>245-download-the-kindle-fire-apk</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>articles/245 - Download the Kindle Fire APK.md</t>
+          <t>245 - Download the Kindle Fire APK.md</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
@@ -11919,12 +11919,12 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/246-overdrive-changelog</t>
+          <t>246-overdrive-changelog</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>articles/246 - OVERDRIVE Changelog.md</t>
+          <t>246 - OVERDRIVE Changelog.md</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
@@ -11952,12 +11952,12 @@
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/247-anki-overdrive-privacy-basics</t>
+          <t>247-anki-overdrive-privacy-basics</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>articles/247 - Anki OVERDRIVE Privacy Basics.md</t>
+          <t>247 - Anki OVERDRIVE Privacy Basics.md</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
@@ -11985,12 +11985,12 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/248-quick-start-guide</t>
+          <t>248-quick-start-guide</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>articles/248 - Quick Start Guide (OverDrive).md</t>
+          <t>248 - Quick Start Guide (OverDrive).md</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
@@ -12018,12 +12018,12 @@
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/249-product-compliance</t>
+          <t>249-product-compliance</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>articles/249 - Product Compliance (OverDrive).md</t>
+          <t>249 - Product Compliance (OverDrive).md</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
@@ -12051,12 +12051,12 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/250-recommended-age</t>
+          <t>250-recommended-age</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>articles/250 - Recommended age.md</t>
+          <t>250 - Recommended age.md</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
@@ -12084,12 +12084,12 @@
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/251-combining-overdrive-and-drive</t>
+          <t>251-combining-overdrive-and-drive</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>articles/251 - Combining OVERDRIVE and DRIVE.md</t>
+          <t>251 - Combining OVERDRIVE and DRIVE.md</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
@@ -12117,12 +12117,12 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/252-do-i-need-the-starter-kit</t>
+          <t>252-do-i-need-the-starter-kit</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>articles/252 - Do I need the Starter Kit.md</t>
+          <t>252 - Do I need the Starter Kit.md</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
@@ -12150,12 +12150,12 @@
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/253-compatible-devices-further-information</t>
+          <t>253-compatible-devices-further-information</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>articles/253 - Compatible Devices - further information.md</t>
+          <t>253 - Compatible Devices - further information.md</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
@@ -12183,12 +12183,12 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/254-anki-drive-end-of-life-eol</t>
+          <t>254-anki-drive-end-of-life-eol</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>articles/254 - DRIVE &amp; OVERDRIVE End-of-Life (EoL).md</t>
+          <t>254 - DRIVE &amp; OVERDRIVE End-of-Life (EoL).md</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
@@ -12216,12 +12216,12 @@
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/255-compatible-devices-anki-overdrive-fast-furious-edition</t>
+          <t>255-compatible-devices-anki-overdrive-fast-furious-edition</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>articles/255 - Compatible Devices - OVERDRIVE - Fast &amp; Furious Edition.md</t>
+          <t>255 - Compatible Devices - OVERDRIVE - Fast &amp; Furious Edition.md</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
@@ -12249,12 +12249,12 @@
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/258-product-disposal-information</t>
+          <t>258-product-disposal-information</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>articles/258 - Product Disposal Information (OverDrive).md</t>
+          <t>258 - Product Disposal Information (OverDrive).md</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
@@ -12282,12 +12282,12 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/264-where-can-i-purchase-tires-and-other-spare-parts</t>
+          <t>264-where-can-i-purchase-tires-and-other-spare-parts</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>articles/264 - Where can I purchase tires and other spare parts.md</t>
+          <t>264 - Where can I purchase tires and other spare parts.md</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
@@ -12315,12 +12315,12 @@
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/265-why-is-scanning-not-successful</t>
+          <t>265-why-is-scanning-not-successful</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>articles/265 - Why is scanning not successful.md</t>
+          <t>265 - Why is scanning not successful.md</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
@@ -12348,12 +12348,12 @@
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/266-video-why-do-my-vehicles-go-off-track</t>
+          <t>266-video-why-do-my-vehicles-go-off-track</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>articles/266 - [VIDEO] Why do my vehicles go off track.md</t>
+          <t>266 - [VIDEO] Why do my vehicles go off track.md</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
@@ -12381,12 +12381,12 @@
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/267-charging-vehicles-and-battery-life</t>
+          <t>267-charging-vehicles-and-battery-life</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>articles/267 - Charging vehicles and battery life.md</t>
+          <t>267 - Charging vehicles and battery life.md</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
@@ -12414,12 +12414,12 @@
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/268-detecting-and-connecting-to-vehicles</t>
+          <t>268-detecting-and-connecting-to-vehicles</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>articles/268 - Detecting and connecting to vehicles.md</t>
+          <t>268 - Detecting and connecting to vehicles.md</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
@@ -12447,12 +12447,12 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/269-multiplayer-requirements-and-troubleshooting</t>
+          <t>269-multiplayer-requirements-and-troubleshooting</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>articles/269 - Multiplayer - requirements and troubleshooting.md</t>
+          <t>269 - Multiplayer - requirements and troubleshooting.md</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
@@ -12480,12 +12480,12 @@
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/270-how-do-i-increase-rank</t>
+          <t>270-how-do-i-increase-rank</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>articles/270 - How do I increase Rank.md</t>
+          <t>270 - How do I increase Rank.md</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
@@ -12513,12 +12513,12 @@
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/271-video-looking-after-your-track-and-vehicles</t>
+          <t>271-video-looking-after-your-track-and-vehicles</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>articles/271 - [VIDEO] Looking after your track and vehicles.md</t>
+          <t>271 - [VIDEO] Looking after your track and vehicles.md</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
@@ -12546,12 +12546,12 @@
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/272-how-to-build-the-best-tracks</t>
+          <t>272-how-to-build-the-best-tracks</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>articles/272 - How to build the best tracks.md</t>
+          <t>272 - How to build the best tracks.md</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
@@ -12579,12 +12579,12 @@
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/273-whats-the-difference-between-experience-points-and-coins</t>
+          <t>273-whats-the-difference-between-experience-points-and-coins</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>articles/273 - What's the difference between Experience Points and Coins.md</t>
+          <t>273 - What's the difference between Experience Points and Coins.md</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
@@ -12612,12 +12612,12 @@
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/274-enabling-location-services</t>
+          <t>274-enabling-location-services</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>articles/274 - Enabling Location Services.md</t>
+          <t>274 - Enabling Location Services.md</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
@@ -12645,12 +12645,12 @@
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/275-how-to-mount-rails</t>
+          <t>275-how-to-mount-rails</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>articles/275 - How to mount Rails.md</t>
+          <t>275 - How to mount Rails.md</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
@@ -12678,12 +12678,12 @@
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/276-what-is-rage-mode</t>
+          <t>276-what-is-rage-mode</t>
         </is>
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>articles/276 - What is Rage mode.md</t>
+          <t>276 - What is Rage mode.md</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
@@ -12711,12 +12711,12 @@
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/277-whats-different-about-supertrucks</t>
+          <t>277-whats-different-about-supertrucks</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>articles/277 - What's different about Supertrucks.md</t>
+          <t>277 - What's different about Supertrucks.md</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
@@ -12744,12 +12744,12 @@
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/278-how-to-play-open-play-modes</t>
+          <t>278-how-to-play-open-play-modes</t>
         </is>
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>articles/278 - How to play Open Play modes.md</t>
+          <t>278 - How to play Open Play modes.md</t>
         </is>
       </c>
       <c r="D101" s="2" t="inlineStr">
@@ -12777,12 +12777,12 @@
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/279-what-is-fire-assist</t>
+          <t>279-what-is-fire-assist</t>
         </is>
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>articles/279 - What is Fire Assist.md</t>
+          <t>279 - What is Fire Assist.md</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr">
@@ -12810,12 +12810,12 @@
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/280-what-do-the-lights-mean</t>
+          <t>280-what-do-the-lights-mean</t>
         </is>
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>articles/280 - What do the lights mean.md</t>
+          <t>280 - What do the lights mean.md</t>
         </is>
       </c>
       <c r="D103" s="2" t="inlineStr">
@@ -12843,12 +12843,12 @@
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/281-overview-of-weapons-range</t>
+          <t>281-overview-of-weapons-range</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>articles/281 - Overview of Weapons' Range.md</t>
+          <t>281 - Overview of Weapons' Range.md</t>
         </is>
       </c>
       <c r="D104" s="2" t="inlineStr">
@@ -12876,12 +12876,12 @@
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/282-the-8-basic-tracks</t>
+          <t>282-the-8-basic-tracks</t>
         </is>
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>articles/282 - The 8 Basic Tracks.md</t>
+          <t>282 - The 8 Basic Tracks.md</t>
         </is>
       </c>
       <c r="D105" s="2" t="inlineStr">
@@ -12909,12 +12909,12 @@
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/283-how-do-i-turn-off-my-vehicle</t>
+          <t>283-how-do-i-turn-off-my-vehicle</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>articles/283 - How do I turn off my vehicle.md</t>
+          <t>283 - How do I turn off my vehicle.md</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
@@ -12942,12 +12942,12 @@
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/284-unlocking-the-power-zone-track-piece</t>
+          <t>284-unlocking-the-power-zone-track-piece</t>
         </is>
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>articles/284 - Unlocking the Power Zone track piece.md</t>
+          <t>284 - Unlocking the Power Zone track piece.md</t>
         </is>
       </c>
       <c r="D107" s="2" t="inlineStr">
@@ -12975,12 +12975,12 @@
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/285-updating-your-anki-overdrive-account</t>
+          <t>285-updating-your-anki-overdrive-account</t>
         </is>
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>articles/285 - Updating your Anki OVERDRIVE account.md</t>
+          <t>285 - Updating your Anki OVERDRIVE account.md</t>
         </is>
       </c>
       <c r="D108" s="2" t="inlineStr">
@@ -13008,12 +13008,12 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/286-what-is-pro-speed</t>
+          <t>286-what-is-pro-speed</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
         <is>
-          <t>articles/286 - What is Pro Speed.md</t>
+          <t>286 - What is Pro Speed.md</t>
         </is>
       </c>
       <c r="D109" s="2" t="inlineStr">
@@ -13041,12 +13041,12 @@
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/287-what-are-racing-lanes</t>
+          <t>287-what-are-racing-lanes</t>
         </is>
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>articles/287 - What are Racing Lanes.md</t>
+          <t>287 - What are Racing Lanes.md</t>
         </is>
       </c>
       <c r="D110" s="2" t="inlineStr">
@@ -13074,12 +13074,12 @@
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/288-how-should-i-store-my-vehicles</t>
+          <t>288-how-should-i-store-my-vehicles</t>
         </is>
       </c>
       <c r="C111" s="2" t="inlineStr">
         <is>
-          <t>articles/288 - How should I store my vehicles.md</t>
+          <t>288 - How should I store my vehicles.md</t>
         </is>
       </c>
       <c r="D111" s="2" t="inlineStr">
@@ -13107,12 +13107,12 @@
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/321-cork-the-volcano</t>
+          <t>321-cork-the-volcano</t>
         </is>
       </c>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>articles/321 - Cork the Volcano.md</t>
+          <t>321 - Cork the Volcano.md</t>
         </is>
       </c>
       <c r="D112" s="2" t="inlineStr">
@@ -13140,12 +13140,12 @@
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/322-abacus-finch</t>
+          <t>322-abacus-finch</t>
         </is>
       </c>
       <c r="C113" s="2" t="inlineStr">
         <is>
-          <t>articles/322 - Abacus Finch.md</t>
+          <t>322 - Abacus Finch.md</t>
         </is>
       </c>
       <c r="D113" s="2" t="inlineStr">
@@ -13173,12 +13173,12 @@
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/323-swatch-out</t>
+          <t>323-swatch-out</t>
         </is>
       </c>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t>articles/323 - Swatch Out.md</t>
+          <t>323 - Swatch Out.md</t>
         </is>
       </c>
       <c r="D114" s="2" t="inlineStr">
@@ -13206,12 +13206,12 @@
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/324-puzzlet-training-portal</t>
+          <t>324-puzzlet-training-portal</t>
         </is>
       </c>
       <c r="C115" s="2" t="inlineStr">
         <is>
-          <t>articles/324 - Puzzlet - Training Portal.md</t>
+          <t>324 - Puzzlet - Training Portal.md</t>
         </is>
       </c>
       <c r="D115" s="2" t="inlineStr">
@@ -13239,12 +13239,12 @@
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/329-overdrive-2-6-frequently-asked-questions</t>
+          <t>329-overdrive-2-6-frequently-asked-questions</t>
         </is>
       </c>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t>articles/329 - OverDrive 2.6 Re-Release - Frequently Asked Questions.md</t>
+          <t>329 - OverDrive 2.6 Re-Release - Frequently Asked Questions.md</t>
         </is>
       </c>
       <c r="D116" s="2" t="inlineStr">
@@ -13272,12 +13272,12 @@
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/330-puzzlet-games-steam</t>
+          <t>330-puzzlet-games-steam</t>
         </is>
       </c>
       <c r="C117" s="2" t="inlineStr">
         <is>
-          <t>articles/330 - Puzzlet Games - Steam.md</t>
+          <t>330 - Puzzlet Games - Steam.md</t>
         </is>
       </c>
       <c r="D117" s="2" t="inlineStr">
@@ -13305,12 +13305,12 @@
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/331-overdrive-2-6-changelog-and-known-issues</t>
+          <t>331-overdrive-2-6-changelog-and-known-issues</t>
         </is>
       </c>
       <c r="C118" s="2" t="inlineStr">
         <is>
-          <t>articles/331 - OverDrive 2.6 - Changelog and Known Issues.md</t>
+          <t>331 - OverDrive 2.6 - Changelog and Known Issues.md</t>
         </is>
       </c>
       <c r="D118" s="2" t="inlineStr">
@@ -13338,12 +13338,12 @@
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/332-introduction-to-puzzlets</t>
+          <t>332-introduction-to-puzzlets</t>
         </is>
       </c>
       <c r="C119" s="2" t="inlineStr">
         <is>
-          <t>articles/332 - Introduction to Puzzlets.md</t>
+          <t>332 - Introduction to Puzzlets.md</t>
         </is>
       </c>
       <c r="D119" s="2" t="inlineStr">
@@ -13371,12 +13371,12 @@
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/333-puzzlets-troubleshooting</t>
+          <t>333-puzzlets-troubleshooting</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>articles/333 - Puzzlets Troubleshooting.md</t>
+          <t>333 - Puzzlets Troubleshooting.md</t>
         </is>
       </c>
       <c r="D120" s="2" t="inlineStr">
@@ -13404,12 +13404,12 @@
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/334-curriculum-and-other-resources</t>
+          <t>334-curriculum-and-other-resources</t>
         </is>
       </c>
       <c r="C121" s="2" t="inlineStr">
         <is>
-          <t>articles/334 - Curriculum and Other Resources.md</t>
+          <t>334 - Curriculum and Other Resources.md</t>
         </is>
       </c>
       <c r="D121" s="2" t="inlineStr">
@@ -13437,12 +13437,12 @@
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/338-how-do-i-find-vectors-serial-number</t>
+          <t>338-how-do-i-find-vectors-serial-number</t>
         </is>
       </c>
       <c r="C122" s="2" t="inlineStr">
         <is>
-          <t>articles/338 - How Do I Find Vector's Serial Number.md</t>
+          <t>338 - How Do I Find Vector's Serial Number.md</t>
         </is>
       </c>
       <c r="D122" s="2" t="inlineStr">
@@ -13470,12 +13470,12 @@
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/341-tire-replacement</t>
+          <t>341-tire-replacement</t>
         </is>
       </c>
       <c r="C123" s="2" t="inlineStr">
         <is>
-          <t>articles/341 - Tire Replacement.md</t>
+          <t>341 - Tire Replacement.md</t>
         </is>
       </c>
       <c r="D123" s="2" t="inlineStr">
@@ -13503,12 +13503,12 @@
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/342-setting-up-vector-with-no-subscription</t>
+          <t>342-setting-up-vector-with-no-subscription</t>
         </is>
       </c>
       <c r="C124" s="2" t="inlineStr">
         <is>
-          <t>articles/342 - Setting Up Vector with No Subscription.md</t>
+          <t>342 - Setting Up Vector with No Subscription.md</t>
         </is>
       </c>
       <c r="D124" s="2" t="inlineStr">
@@ -13536,12 +13536,12 @@
       </c>
       <c r="B125" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/344-all-about-memberships</t>
+          <t>344-all-about-memberships</t>
         </is>
       </c>
       <c r="C125" s="2" t="inlineStr">
         <is>
-          <t>articles/344 - All About Vector Memberships.md</t>
+          <t>344 - All About Vector Memberships.md</t>
         </is>
       </c>
       <c r="D125" s="2" t="inlineStr">
@@ -13569,12 +13569,12 @@
       </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/349-escape-pod-robot-onboarding-oskr</t>
+          <t>349-escape-pod-robot-onboarding-oskr</t>
         </is>
       </c>
       <c r="C126" s="2" t="inlineStr">
         <is>
-          <t>articles/349 - OSKR Users - Robot Onboarding for Escape Pod.md</t>
+          <t>349 - OSKR Users - Robot Onboarding for Escape Pod.md</t>
         </is>
       </c>
       <c r="D126" s="2" t="inlineStr">
@@ -13602,12 +13602,12 @@
       </c>
       <c r="B127" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/350-oskr-users-pi-flashing-for-the-escape-pod</t>
+          <t>350-oskr-users-pi-flashing-for-the-escape-pod</t>
         </is>
       </c>
       <c r="C127" s="2" t="inlineStr">
         <is>
-          <t>articles/350 - OSKR Users - Pi Flashing for the Escape Pod.md</t>
+          <t>350 - OSKR Users - Pi Flashing for the Escape Pod.md</t>
         </is>
       </c>
       <c r="D127" s="2" t="inlineStr">
@@ -13635,12 +13635,12 @@
       </c>
       <c r="B128" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/351-known-issues</t>
+          <t>351-known-issues</t>
         </is>
       </c>
       <c r="C128" s="2" t="inlineStr">
         <is>
-          <t>articles/351 - Escape Pod - Changelog, Limitations &amp; Known Issues.md</t>
+          <t>351 - Escape Pod - Changelog, Limitations &amp; Known Issues.md</t>
         </is>
       </c>
       <c r="D128" s="2" t="inlineStr">
@@ -13668,12 +13668,12 @@
       </c>
       <c r="B129" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/352-oskr-users-returning-to-ddl-server</t>
+          <t>352-oskr-users-returning-to-ddl-server</t>
         </is>
       </c>
       <c r="C129" s="2" t="inlineStr">
         <is>
-          <t>articles/352 - OSKR Users - Returning to DDL Server.md</t>
+          <t>352 - OSKR Users - Returning to DDL Server.md</t>
         </is>
       </c>
       <c r="D129" s="2" t="inlineStr">
@@ -13701,12 +13701,12 @@
       </c>
       <c r="B130" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/355-launching-your-escape-pod</t>
+          <t>355-launching-your-escape-pod</t>
         </is>
       </c>
       <c r="C130" s="2" t="inlineStr">
         <is>
-          <t>articles/355 - Launching Your Escape Pod, Step 1 - Assemble Your Pi Kit.md</t>
+          <t>355 - Launching Your Escape Pod, Step 1 - Assemble Your Pi Kit.md</t>
         </is>
       </c>
       <c r="D130" s="2" t="inlineStr">
@@ -13734,12 +13734,12 @@
       </c>
       <c r="B131" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/357-returning-to-ddl-server</t>
+          <t>357-returning-to-ddl-server</t>
         </is>
       </c>
       <c r="C131" s="2" t="inlineStr">
         <is>
-          <t>articles/357 - Returning to DDL Server.md</t>
+          <t>357 - Returning to DDL Server.md</t>
         </is>
       </c>
       <c r="D131" s="2" t="inlineStr">
@@ -13767,12 +13767,12 @@
       </c>
       <c r="B132" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/358-launching-your-escape-pod-2</t>
+          <t>358-launching-your-escape-pod-2</t>
         </is>
       </c>
       <c r="C132" s="2" t="inlineStr">
         <is>
-          <t>articles/358 - Launching Your Escape Pod, Step 2 - Flash The SD Card.md</t>
+          <t>358 - Launching Your Escape Pod, Step 2 - Flash The SD Card.md</t>
         </is>
       </c>
       <c r="D132" s="2" t="inlineStr">
@@ -13800,12 +13800,12 @@
       </c>
       <c r="B133" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/359-launching-your-escape-pod-3</t>
+          <t>359-launching-your-escape-pod-3</t>
         </is>
       </c>
       <c r="C133" s="2" t="inlineStr">
         <is>
-          <t>articles/359 - Launching Your Escape Pod, Step 3 - Connecting The Escape Pod.md</t>
+          <t>359 - Launching Your Escape Pod, Step 3 - Connecting The Escape Pod.md</t>
         </is>
       </c>
       <c r="D133" s="2" t="inlineStr">
@@ -13833,12 +13833,12 @@
       </c>
       <c r="B134" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/360-launching-your-escape-pod-4</t>
+          <t>360-launching-your-escape-pod-4</t>
         </is>
       </c>
       <c r="C134" s="2" t="inlineStr">
         <is>
-          <t>articles/360 - Launching Your Escape Pod, Step 4 - Onboarding Your Vector Robot.md</t>
+          <t>360 - Launching Your Escape Pod, Step 4 - Onboarding Your Vector Robot.md</t>
         </is>
       </c>
       <c r="D134" s="2" t="inlineStr">
@@ -13866,12 +13866,12 @@
       </c>
       <c r="B135" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/361-vector-developer-tools</t>
+          <t>361-vector-developer-tools</t>
         </is>
       </c>
       <c r="C135" s="2" t="inlineStr">
         <is>
-          <t>articles/361 - Vector Developer Tools.md</t>
+          <t>361 - Vector Developer Tools.md</t>
         </is>
       </c>
       <c r="D135" s="2" t="inlineStr">
@@ -13899,12 +13899,12 @@
       </c>
       <c r="B136" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/363-escape-pod-ssh-access-logging</t>
+          <t>363-escape-pod-ssh-access-logging</t>
         </is>
       </c>
       <c r="C136" s="2" t="inlineStr">
         <is>
-          <t>articles/363 - SSH Access &amp; Logging.md</t>
+          <t>363 - SSH Access &amp; Logging.md</t>
         </is>
       </c>
       <c r="D136" s="2" t="inlineStr">
@@ -13932,12 +13932,12 @@
       </c>
       <c r="B137" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/371-multiple-vectors-on-escape-pod</t>
+          <t>371-multiple-vectors-on-escape-pod</t>
         </is>
       </c>
       <c r="C137" s="2" t="inlineStr">
         <is>
-          <t>articles/371 - Managing Multiple Vectors on Escape Pod.md</t>
+          <t>371 - Managing Multiple Vectors on Escape Pod.md</t>
         </is>
       </c>
       <c r="D137" s="2" t="inlineStr">
@@ -13965,12 +13965,12 @@
       </c>
       <c r="B138" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/372-switching-views-on-escape-pod</t>
+          <t>372-switching-views-on-escape-pod</t>
         </is>
       </c>
       <c r="C138" s="2" t="inlineStr">
         <is>
-          <t>articles/372 - Using the Terminal on Escape Pod.md</t>
+          <t>372 - Using the Terminal on Escape Pod.md</t>
         </is>
       </c>
       <c r="D138" s="2" t="inlineStr">
@@ -13998,12 +13998,12 @@
       </c>
       <c r="B139" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/373-claiming-your-15-canakit-rebate</t>
+          <t>373-claiming-your-15-canakit-rebate</t>
         </is>
       </c>
       <c r="C139" s="2" t="inlineStr">
         <is>
-          <t>articles/373 - Claiming Your $15 CanaKit Rebate.md</t>
+          <t>373 - Claiming Your $15 CanaKit Rebate.md</t>
         </is>
       </c>
       <c r="D139" s="2" t="inlineStr">
@@ -14031,12 +14031,12 @@
       </c>
       <c r="B140" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/374-escape-pod-command-line-commands</t>
+          <t>374-escape-pod-command-line-commands</t>
         </is>
       </c>
       <c r="C140" s="2" t="inlineStr">
         <is>
-          <t>articles/374 - Command Line - Commands &amp; Options.md</t>
+          <t>374 - Command Line - Commands &amp; Options.md</t>
         </is>
       </c>
       <c r="D140" s="2" t="inlineStr">
@@ -14064,12 +14064,12 @@
       </c>
       <c r="B141" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/376-onboarding-no-devices-found-error</t>
+          <t>376-onboarding-no-devices-found-error</t>
         </is>
       </c>
       <c r="C141" s="2" t="inlineStr">
         <is>
-          <t>articles/376 - Onboarding - No Devices Found Error.md</t>
+          <t>376 - Onboarding - No Devices Found Error.md</t>
         </is>
       </c>
       <c r="D141" s="2" t="inlineStr">
@@ -14097,12 +14097,12 @@
       </c>
       <c r="B142" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/377-firmware-downgrade-not-allowed-error</t>
+          <t>377-firmware-downgrade-not-allowed-error</t>
         </is>
       </c>
       <c r="C142" s="2" t="inlineStr">
         <is>
-          <t>articles/377 - Firmware Loading - Downgrade Not Allowed Error.md</t>
+          <t>377 - Firmware Loading - Downgrade Not Allowed Error.md</t>
         </is>
       </c>
       <c r="D142" s="2" t="inlineStr">
@@ -14130,12 +14130,12 @@
       </c>
       <c r="B143" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/378-onboarding-cant-add-new-device-error</t>
+          <t>378-onboarding-cant-add-new-device-error</t>
         </is>
       </c>
       <c r="C143" s="2" t="inlineStr">
         <is>
-          <t>articles/378 - Onboarding - Can't Add New Device Error.md</t>
+          <t>378 - Onboarding - Can't Add New Device Error.md</t>
         </is>
       </c>
       <c r="D143" s="2" t="inlineStr">
@@ -14163,12 +14163,12 @@
       </c>
       <c r="B144" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/380-turning-vector-on-or-off</t>
+          <t>380-turning-vector-on-or-off</t>
         </is>
       </c>
       <c r="C144" s="2" t="inlineStr">
         <is>
-          <t>articles/380 - Turning Vector On or Off.md</t>
+          <t>380 - Turning Vector On or Off.md</t>
         </is>
       </c>
       <c r="D144" s="2" t="inlineStr">
@@ -14196,12 +14196,12 @@
       </c>
       <c r="B145" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/383-performing-a-firmware-recovery-reset</t>
+          <t>383-performing-a-firmware-recovery-reset</t>
         </is>
       </c>
       <c r="C145" s="2" t="inlineStr">
         <is>
-          <t>articles/383 - Performing a Firmware Recovery Reset.md</t>
+          <t>383 - Performing a Firmware Recovery Reset.md</t>
         </is>
       </c>
       <c r="D145" s="2" t="inlineStr">
@@ -14229,12 +14229,12 @@
       </c>
       <c r="B146" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/384-performing-a-clear-user-data-reset</t>
+          <t>384-performing-a-clear-user-data-reset</t>
         </is>
       </c>
       <c r="C146" s="2" t="inlineStr">
         <is>
-          <t>articles/384 - Performing a Clear User Data Reset.md</t>
+          <t>384 - Performing a Clear User Data Reset.md</t>
         </is>
       </c>
       <c r="D146" s="2" t="inlineStr">
@@ -14262,12 +14262,12 @@
       </c>
       <c r="B147" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/385-community-guidelines</t>
+          <t>385-community-guidelines</t>
         </is>
       </c>
       <c r="C147" s="2" t="inlineStr">
         <is>
-          <t>articles/385 - Community Guidelines.md</t>
+          <t>385 - Community Guidelines.md</t>
         </is>
       </c>
       <c r="D147" s="2" t="inlineStr">
@@ -14295,12 +14295,12 @@
       </c>
       <c r="B148" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/387-cant-reach-digital-dream-labs-error</t>
+          <t>387-cant-reach-digital-dream-labs-error</t>
         </is>
       </c>
       <c r="C148" s="2" t="inlineStr">
         <is>
-          <t>articles/387 - Can't Reach Digital Dream Labs Error.md</t>
+          <t>387 - Can't Reach Digital Dream Labs Error.md</t>
         </is>
       </c>
       <c r="D148" s="2" t="inlineStr">
@@ -14328,12 +14328,12 @@
       </c>
       <c r="B149" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/411-feature-fridays</t>
+          <t>411-feature-fridays</t>
         </is>
       </c>
       <c r="C149" s="2" t="inlineStr">
         <is>
-          <t>articles/411 - Feature Fridays!.md</t>
+          <t>411 - Feature Fridays!.md</t>
         </is>
       </c>
       <c r="D149" s="2" t="inlineStr">
@@ -14361,12 +14361,12 @@
       </c>
       <c r="B150" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/412-cozmo-transferring-code-lab-projects</t>
+          <t>412-cozmo-transferring-code-lab-projects</t>
         </is>
       </c>
       <c r="C150" s="2" t="inlineStr">
         <is>
-          <t>articles/412 - Migrating to Cozmo App Version 3.4.1 and Above.md</t>
+          <t>412 - Migrating to Cozmo App Version 3.4.1 and Above.md</t>
         </is>
       </c>
       <c r="D150" s="2" t="inlineStr">
@@ -14394,12 +14394,12 @@
       </c>
       <c r="B151" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/413-changing-vectors-eye-color</t>
+          <t>413-changing-vectors-eye-color</t>
         </is>
       </c>
       <c r="C151" s="2" t="inlineStr">
         <is>
-          <t>articles/413 - Changing Vector's Eye Color.md</t>
+          <t>413 - Changing Vector's Eye Color.md</t>
         </is>
       </c>
       <c r="D151" s="2" t="inlineStr">
@@ -14427,12 +14427,12 @@
       </c>
       <c r="B152" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/417-age-requirement-error-message</t>
+          <t>417-age-requirement-error-message</t>
         </is>
       </c>
       <c r="C152" s="2" t="inlineStr">
         <is>
-          <t>articles/417 - Age Requirement Error Message.md</t>
+          <t>417 - Age Requirement Error Message.md</t>
         </is>
       </c>
       <c r="D152" s="2" t="inlineStr">
@@ -14460,12 +14460,12 @@
       </c>
       <c r="B153" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/467-vector-already-has-an-owner</t>
+          <t>467-vector-already-has-an-owner</t>
         </is>
       </c>
       <c r="C153" s="2" t="inlineStr">
         <is>
-          <t>articles/467 - This Vector Already Has An Owner Error Message.md</t>
+          <t>467 - This Vector Already Has An Owner Error Message.md</t>
         </is>
       </c>
       <c r="D153" s="2" t="inlineStr">
@@ -14493,12 +14493,12 @@
       </c>
       <c r="B154" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/468-onboarding-authorization-failed-error</t>
+          <t>468-onboarding-authorization-failed-error</t>
         </is>
       </c>
       <c r="C154" s="2" t="inlineStr">
         <is>
-          <t>articles/468 - Onboarding - Authorization Failed Error.md</t>
+          <t>468 - Onboarding - Authorization Failed Error.md</t>
         </is>
       </c>
       <c r="D154" s="2" t="inlineStr">
@@ -14526,12 +14526,12 @@
       </c>
       <c r="B155" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/474-vector-app-cant-find-vector-via-bluetooth</t>
+          <t>474-vector-app-cant-find-vector-via-bluetooth</t>
         </is>
       </c>
       <c r="C155" s="2" t="inlineStr">
         <is>
-          <t>articles/474 - Vector App Can't Find Vector via Bluetooth.md</t>
+          <t>474 - Vector App Can't Find Vector via Bluetooth.md</t>
         </is>
       </c>
       <c r="D155" s="2" t="inlineStr">
@@ -14559,12 +14559,12 @@
       </c>
       <c r="B156" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/475-enabling-bluetooth-on-your-device</t>
+          <t>475-enabling-bluetooth-on-your-device</t>
         </is>
       </c>
       <c r="C156" s="2" t="inlineStr">
         <is>
-          <t>articles/475 - Enabling Bluetooth On Your Device.md</t>
+          <t>475 - Enabling Bluetooth On Your Device.md</t>
         </is>
       </c>
       <c r="D156" s="2" t="inlineStr">
@@ -14592,12 +14592,12 @@
       </c>
       <c r="B157" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/476-enabling-wi-fi-on-your-device</t>
+          <t>476-enabling-wi-fi-on-your-device</t>
         </is>
       </c>
       <c r="C157" s="2" t="inlineStr">
         <is>
-          <t>articles/476 - Enabling Wi-Fi On Your Device.md</t>
+          <t>476 - Enabling Wi-Fi On Your Device.md</t>
         </is>
       </c>
       <c r="D157" s="2" t="inlineStr">
@@ -14625,12 +14625,12 @@
       </c>
       <c r="B158" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/477-creating-a-2-4ghz-network</t>
+          <t>477-creating-a-2-4ghz-network</t>
         </is>
       </c>
       <c r="C158" s="2" t="inlineStr">
         <is>
-          <t>articles/477 - Creating a 2.4GHz Network.md</t>
+          <t>477 - Creating a 2.4GHz Network.md</t>
         </is>
       </c>
       <c r="D158" s="2" t="inlineStr">
@@ -14658,12 +14658,12 @@
       </c>
       <c r="B159" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/479-vector-is-syncing</t>
+          <t>479-vector-is-syncing</t>
         </is>
       </c>
       <c r="C159" s="2" t="inlineStr">
         <is>
-          <t>articles/479 - Vector Is Syncing Error Message.md</t>
+          <t>479 - Vector Is Syncing Error Message.md</t>
         </is>
       </c>
       <c r="D159" s="2" t="inlineStr">
@@ -14691,12 +14691,12 @@
       </c>
       <c r="B160" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/480-activate-your-ddl-account</t>
+          <t>480-activate-your-ddl-account</t>
         </is>
       </c>
       <c r="C160" s="2" t="inlineStr">
         <is>
-          <t>articles/480 - Activate Your Digital Dream Labs Account.md</t>
+          <t>480 - Activate Your Digital Dream Labs Account.md</t>
         </is>
       </c>
       <c r="D160" s="2" t="inlineStr">
@@ -14724,12 +14724,12 @@
       </c>
       <c r="B161" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/504-all-about-lifetime-licenses</t>
+          <t>504-all-about-lifetime-licenses</t>
         </is>
       </c>
       <c r="C161" s="2" t="inlineStr">
         <is>
-          <t>articles/504 - All About Lifetime Licenses.md</t>
+          <t>504 - All About Lifetime Licenses.md</t>
         </is>
       </c>
       <c r="D161" s="2" t="inlineStr">
@@ -14757,12 +14757,12 @@
       </c>
       <c r="B162" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/513-state-of-manufacturing-butter-robot</t>
+          <t>513-state-of-manufacturing-butter-robot</t>
         </is>
       </c>
       <c r="C162" s="2" t="inlineStr">
         <is>
-          <t>articles/513 - State of Manufacturing - Butter Robot.md</t>
+          <t>513 - State of Manufacturing - Butter Robot.md</t>
         </is>
       </c>
       <c r="D162" s="2" t="inlineStr">
@@ -14790,12 +14790,12 @@
       </c>
       <c r="B163" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/515-state-of-manufacturing-cozmo-2-0</t>
+          <t>515-state-of-manufacturing-cozmo-2-0</t>
         </is>
       </c>
       <c r="C163" s="2" t="inlineStr">
         <is>
-          <t>articles/515 - State of Manufacturing - Cozmo 2.0.md</t>
+          <t>515 - State of Manufacturing - Cozmo 2.0.md</t>
         </is>
       </c>
       <c r="D163" s="2" t="inlineStr">
@@ -14823,12 +14823,12 @@
       </c>
       <c r="B164" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/516-state-of-manufacturing-vector-2-0</t>
+          <t>516-state-of-manufacturing-vector-2-0</t>
         </is>
       </c>
       <c r="C164" s="2" t="inlineStr">
         <is>
-          <t>articles/516 - State of Manufacturing - Vector 2.0.md</t>
+          <t>516 - State of Manufacturing - Vector 2.0.md</t>
         </is>
       </c>
       <c r="D164" s="2" t="inlineStr">
@@ -14856,12 +14856,12 @@
       </c>
       <c r="B165" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/519-escapepod-transferring-behaviors</t>
+          <t>519-escapepod-transferring-behaviors</t>
         </is>
       </c>
       <c r="C165" s="2" t="inlineStr">
         <is>
-          <t>articles/519 - Transferring Customized Commands (Behaviors).md</t>
+          <t>519 - Transferring Customized Commands (Behaviors).md</t>
         </is>
       </c>
       <c r="D165" s="2" t="inlineStr">
@@ -14889,12 +14889,12 @@
       </c>
       <c r="B166" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/520-robot-repair-process</t>
+          <t>520-robot-repair-process</t>
         </is>
       </c>
       <c r="C166" s="2" t="inlineStr">
         <is>
-          <t>articles/520 - Repair Process - Cozmo &amp; Vector.md</t>
+          <t>520 - Repair Process - Cozmo &amp; Vector.md</t>
         </is>
       </c>
       <c r="D166" s="2" t="inlineStr">
@@ -14922,12 +14922,12 @@
       </c>
       <c r="B167" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/522-tracking-your-repair</t>
+          <t>522-tracking-your-repair</t>
         </is>
       </c>
       <c r="C167" s="2" t="inlineStr">
         <is>
-          <t>articles/522 - Tracking Your Repair.md</t>
+          <t>522 - Tracking Your Repair.md</t>
         </is>
       </c>
       <c r="D167" s="2" t="inlineStr">
@@ -14955,12 +14955,12 @@
       </c>
       <c r="B168" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/523-collecting-logs-vector</t>
+          <t>523-collecting-logs-vector</t>
         </is>
       </c>
       <c r="C168" s="2" t="inlineStr">
         <is>
-          <t>articles/523 - Collecting Logs from Vector.md</t>
+          <t>523 - Collecting Logs from Vector.md</t>
         </is>
       </c>
       <c r="D168" s="2" t="inlineStr">
@@ -14988,12 +14988,12 @@
       </c>
       <c r="B169" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/531-vector-ccis</t>
+          <t>531-vector-ccis</t>
         </is>
       </c>
       <c r="C169" s="2" t="inlineStr">
         <is>
-          <t>articles/531 - The Customer Care Information Screen.md</t>
+          <t>531 - The Customer Care Information Screen.md</t>
         </is>
       </c>
       <c r="D169" s="2" t="inlineStr">
@@ -15021,12 +15021,12 @@
       </c>
       <c r="B170" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/532-update-your-shipping-address</t>
+          <t>532-update-your-shipping-address</t>
         </is>
       </c>
       <c r="C170" s="2" t="inlineStr">
         <is>
-          <t>articles/532 - Update Your Shipping Address.md</t>
+          <t>532 - Update Your Shipping Address.md</t>
         </is>
       </c>
       <c r="D170" s="2" t="inlineStr">
@@ -15054,12 +15054,12 @@
       </c>
       <c r="B171" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/254-anki-overdrive-end-of-life-eol</t>
+          <t>254-anki-overdrive-end-of-life-eol</t>
         </is>
       </c>
       <c r="C171" s="2" t="inlineStr">
         <is>
-          <t>articles/254 - DRIVE &amp; OVERDRIVE End-of-Life (EoL).md</t>
+          <t>254 - DRIVE &amp; OVERDRIVE End-of-Life (EoL).md</t>
         </is>
       </c>
       <c r="D171" s="2" t="inlineStr">
@@ -15079,7 +15079,7 @@
       </c>
       <c r="G171" s="2" t="inlineStr">
         <is>
-          <t>Byte-identical duplicate of 'support.digitaldreamlabs.com/article/254-anki-drive-end-of-life-eol' - collapsed into the single file above</t>
+          <t>Byte-identical duplicate of '254-anki-drive-end-of-life-eol' - collapsed into the single file above</t>
         </is>
       </c>
     </row>
@@ -15091,12 +15091,12 @@
       </c>
       <c r="B172" s="2" t="inlineStr">
         <is>
-          <t>support.digitaldreamlabs.com/article/255-compatible-devices-overdrive-fast-furious-edition</t>
+          <t>255-compatible-devices-overdrive-fast-furious-edition</t>
         </is>
       </c>
       <c r="C172" s="2" t="inlineStr">
         <is>
-          <t>articles/255 - Compatible Devices - OVERDRIVE - Fast &amp; Furious Edition.md</t>
+          <t>255 - Compatible Devices - OVERDRIVE - Fast &amp; Furious Edition.md</t>
         </is>
       </c>
       <c r="D172" s="2" t="inlineStr">
@@ -15116,7 +15116,7 @@
       </c>
       <c r="G172" s="2" t="inlineStr">
         <is>
-          <t>Byte-identical duplicate of 'support.digitaldreamlabs.com/article/255-compatible-devices-anki-overdrive-fast-furious-edition' - collapsed into the single file above</t>
+          <t>Byte-identical duplicate of '255-compatible-devices-anki-overdrive-fast-furious-edition' - collapsed into the single file above</t>
         </is>
       </c>
     </row>

</xml_diff>